<commit_message>
publish site with 27.07 forecast
</commit_message>
<xml_diff>
--- a/Grafik_CCEE_SLIVEN1_28_07_2026.xlsx
+++ b/Grafik_CCEE_SLIVEN1_28_07_2026.xlsx
@@ -1827,8 +1827,10 @@
       <c r="B58" s="1" t="n">
         <v>46231</v>
       </c>
-      <c r="C58" s="11" t="n">
-        <v>0</v>
+      <c r="C58" s="10" t="inlineStr">
+        <is>
+          <t>Put Adex Solcast value here</t>
+        </is>
       </c>
       <c r="D58" s="5" t="n">
         <v>0</v>
@@ -2147,10 +2149,8 @@
       <c r="B74" s="1" t="n">
         <v>46231</v>
       </c>
-      <c r="C74" s="10" t="inlineStr">
-        <is>
-          <t>Put Adex Solcast value here</t>
-        </is>
+      <c r="C74" s="11" t="n">
+        <v>0</v>
       </c>
       <c r="D74" s="5" t="n">
         <v>0</v>

</xml_diff>